<commit_message>
Display CLXN with former EFCAB1 name in author decision workbook
</commit_message>
<xml_diff>
--- a/outputs/temporal-author-cutoff-decisions-20261019/Temporal_Case_Author_Decisions_Cutoff_20261019.xlsx
+++ b/outputs/temporal-author-cutoff-decisions-20261019/Temporal_Case_Author_Decisions_Cutoff_20261019.xlsx
@@ -4482,8 +4482,10 @@
       </c>
     </row>
     <row r="22" spans="1:11" ht="114" customHeight="1">
-      <c r="A22" s="28" t="s">
-        <v>708</v>
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CLXN (formerly EFCAB1)</t>
+        </is>
       </c>
       <c r="B22" s="2" t="s">
         <v>710</v>
@@ -5859,7 +5861,7 @@
     <hyperlink ref="A24" location="'Evidence'!A249" display="GPATCH11" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
     <hyperlink ref="A23" location="'Evidence'!A232" display="FSD1L" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
     <hyperlink ref="A21" location="'Evidence'!A200" display="DNAJC30" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="A22" location="'Evidence'!A216" display="EFCAB1" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="A22" location="'Evidence'!A216" display="CLXN (formerly EFCAB1)" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -7521,8 +7523,10 @@
       <c r="B215" s="2"/>
     </row>
     <row r="216" spans="1:2" ht="26" customHeight="1">
-      <c r="A216" s="1" t="s">
-        <v>708</v>
+      <c r="A216" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CLXN (formerly EFCAB1)</t>
+        </is>
       </c>
       <c r="B216" s="1" t="s">
         <v>194</v>
@@ -15573,7 +15577,7 @@
         </is>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="48" customHeight="1">
+    <row r="16" spans="1:4" ht="68" customHeight="1">
       <c r="A16" s="10" t="s">
         <v>48</v>
       </c>
@@ -15583,8 +15587,10 @@
       <c r="C16" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="10" t="s">
-        <v>51</v>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CLXN (formerly EFCAB1) is the current display for HGNC:25678. The original TSV and returned files retain their historical symbol. HGNC: https://rest.genenames.org/fetch/hgnc_id/25678</t>
+        </is>
       </c>
     </row>
     <row r="17" spans="1:4" ht="48" customHeight="1">

</xml_diff>